<commit_message>
expand knowledge collaboration platform and bug catalog
</commit_message>
<xml_diff>
--- a/report-knowledge-asset-collaboration.xlsx
+++ b/report-knowledge-asset-collaboration.xlsx
@@ -10,7 +10,7 @@
     <sheet name="bug inventory" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'bug inventory'!$A$1:$K$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'bug inventory'!$A$1:$K$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1055,8 +1055,878 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>When a user cancels an annotation request, the annotation service must return context.Canceled and must not create a partial annotation.</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>中文根因：服务必须在创建前检查上下文，取消请求不能继续生成批注。生产文件/符号：internal/annotation/annotation.go:Create。失效原因：客户端断开后若仍写入批注，会产生无作者或无效范围的孤儿批注。证据：Create 接收 context 并执行持久化前校验。 生产文件/符号：internal/annotation.Create 调用链：HTTP/业务服务 → internal/annotation.Create。失效原因：客户端断开后若仍写入批注，会产生无作者或无效范围的孤儿批注。证据：Create 接收 context 并执行持久化前校验。 证据：Create 接收 context 并执行持久化前校验。</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>目标行为：取消上下文不创建批注。边界：取消发生在调用前；非法范围也必须拒绝。合法场景：有效范围和有效正文创建成功。验证标准：错误为 context.Canceled 且成功场景返回带 ID 的批注。</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-011/regression -count=1
+go test -race ./cases/bug-011/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>bug011_green</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>bug011_red</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Completing an attachment must reject unknown attachment IDs and preserve the original upload state.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>中文根因：附件完成接口需要区分不存在资源和正常完成。生产文件/符号：internal/attachment/service.go:Service.Complete。失效原因：调用方把重试请求当成成功会导致下载列表显示不完整附件。证据：Complete 读取 items 后更新 Uploaded 字段。 生产文件/符号：internal/attachment.Service.Complete 调用链：HTTP/业务服务 → internal/attachment.Service.Complete。失效原因：调用方把重试请求当成成功会导致下载列表显示不完整附件。证据：Complete 读取 items 后更新 Uploaded 字段。 证据：Complete 读取 items 后更新 Uploaded 字段。</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>目标行为：未知 ID 返回明确错误；已存在附件完成后 Uploaded 等于 Size。边界：大小为零和重复完成都不能破坏状态。合法场景：已启动分片附件可以完成。验证标准：错误非 nil，完成结果 Uploaded==Size，重复完成保持幂等。</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-012/regression -count=1
+go test -race ./cases/bug-012/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>bug012_green</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>bug012_red</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>diagnosis</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>slice</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Audit log listing must return an isolated snapshot so callers cannot mutate historical events.</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>中文根因：审计查询返回值必须与内部事件存储隔离。生产文件/符号：internal/audit/logger.go:Logger.List。失效原因：外部修改返回切片会篡改后续审计查询结果。证据：List 复制切片但事件字段仍需保持不可变语义。 生产文件/符号：internal/audit.Logger.List 调用链：HTTP/业务服务 → internal/audit.Logger.List。失效原因：外部修改返回切片会篡改后续审计查询结果。证据：List 复制切片但事件字段仍需保持不可变语义。 证据：List 复制切片但事件字段仍需保持不可变语义。</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>目标行为：查询结果修改不影响日志存储。边界：空日志返回空切片而非异常。合法场景：多条日志按写入顺序可查询。验证标准：修改第一次查询结果后，第二次查询仍保留原始 ActorID 和 Action。</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-013/regression -count=1
+go test -race ./cases/bug-013/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>bug013_green</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>bug013_red</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Resolving a comment must fail for an unknown comment and must persist the resolved flag for a known comment.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>中文根因：评论解决操作必须校验评论存在性后再写回。生产文件/符号：internal/comment/repository.go:Repository.Resolve。失效原因：未知评论被当成成功会让前端显示虚假的解决状态。证据：Resolve 通过 map 查找评论并更新 Resolved。 生产文件/符号：internal/comment.Repository.Resolve 调用链：HTTP/业务服务 → internal/comment.Repository.Resolve。失效原因：未知评论被当成成功会让前端显示虚假的解决状态。证据：Resolve 通过 map 查找评论并更新 Resolved。 证据：Resolve 通过 map 查找评论并更新 Resolved。</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>目标行为：未知评论返回 not found；已存在评论可解决和重新打开。边界：同一评论重复设置同一状态应幂等。合法场景：作者或管理员操作已有评论。验证标准：错误包含 not found，合法操作后状态可被后续读取或通过未读统计反映。</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-014/regression -count=1
+go test -race ./cases/bug-014/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>bug014_green</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>bug014_red</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Concurrent editor presence updates must retain all distinct users in the document room.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>中文根因：协作房间加入操作必须在共享房间锁内完成。生产文件/符号：internal/editor/hub.go:Hub.Join。失效原因：并发加入若覆盖房间 map，会造成在线用户列表丢失。证据：Join 创建房间并写入用户 presence。 生产文件/符号：internal/editor.Hub.Join 调用链：HTTP/业务服务 → internal/editor.Hub.Join。失效原因：并发加入若覆盖房间 map，会造成在线用户列表丢失。证据：Join 创建房间并写入用户 presence。 证据：Join 创建房间并写入用户 presence。</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>目标行为：并发加入不同用户后 Online 返回全部用户。边界：同一用户重复加入只保留一个 presence。合法场景：多人同时打开同一文档。验证标准：race 测试无数据竞争，用户集合大小和成员均正确。</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-015/regression -count=1
+go test -race ./cases/bug-015/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>bug015_green</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>bug015_red</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Saving a document after request cancellation must return the cancellation error and keep the previous version.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>中文根因：文档草稿保存需要在写锁前后都尊重请求取消。生产文件/符号：internal/document/repository.go:Repository.Save。失效原因：取消请求仍推进版本会让编辑器发生不可恢复的版本冲突。证据：Save 使用 expected version并更新 Body、Version。 生产文件/符号：internal/document.Repository.Save 调用链：HTTP/业务服务 → internal/document.Repository.Save。失效原因：取消请求仍推进版本会让编辑器发生不可恢复的版本冲突。证据：Save 使用 expected version并更新 Body、Version。 证据：Save 使用 expected version并更新 Body、Version。</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>目标行为：取消保存不改变正文和版本。边界：取消前的有效保存仍可成功；错误版本返回乐观锁冲突。合法场景：版本号匹配且上下文有效时保存成功。验证标准：取消调用返回 context.Canceled，随后读取仍为原版本。</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-016/regression -count=1
+go test -race ./cases/bug-016/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>bug016_green</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>bug016_red</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>nil</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Workspace creation must reject a nil context instead of panicking.</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>中文根因：公共服务方法必须把 nil context 视为无效请求。生产文件/符号：internal/workspace/workspace.go:Create。失效原因：后台任务传入 nil 会触发 ctx.Err() 空指针崩溃。证据：Create 直接访问 ctx.Err。 生产文件/符号：internal/workspace.Create 调用链：HTTP/业务服务 → internal/workspace.Create。失效原因：后台任务传入 nil 会触发 ctx.Err() 空指针崩溃。证据：Create 直接访问 ctx.Err。 证据：Create 直接访问 ctx.Err。</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>目标行为：nil context返回错误而不 panic。边界：已取消 context同样返回取消错误。合法场景：context.Background可创建非空名称空间。验证标准：测试使用 recover 确认无 panic，并校验有效调用返回 workspace ID。</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-017/regression -count=1
+go test -race ./cases/bug-017/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>bug017_green</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>bug017_red</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>diagnosis</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>slice</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Permission evaluation must honor an explicit deny even when a broader allow grant exists.</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>中文根因：权限决策需要按显式拒绝优先于继承允许。生产文件/符号：internal/permission/service.go:Service.Allowed。失效原因：同一用户既有全局允许又有文档拒绝时，若顺序依赖会越权。证据：Allowed遍历 grants并处理 ExplicitDeny。 生产文件/符号：internal/permission.Service.Allowed 调用链：HTTP/业务服务 → internal/permission.Service.Allowed。失效原因：同一用户既有全局允许又有文档拒绝时，若顺序依赖会越权。证据：Allowed遍历 grants并处理 ExplicitDeny。 证据：Allowed遍历 grants并处理 ExplicitDeny。</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>目标行为：显式拒绝始终优先。边界：仅有允许时返回 true，仅有拒绝时返回 false。合法场景：用户拥有空间继承允许但文档显式拒绝。验证标准：不同 grant 添加顺序得到相同拒绝结果。</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-018/regression -count=1
+go test -race ./cases/bug-018/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>bug018_green</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>bug018_red</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Creating a share link with a non-positive TTL must return a validation error.</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>中文根因：公开分享必须限制有效期，不能创建立即过期或永久无期限链接。生产文件/符号：internal/share/share.go:Create。失效原因：非正 TTL 会生成不可用分享或绕过平台的过期策略。证据：Create 根据 ttl 计算 ExpiresAt。 生产文件/符号：internal/share.Create 调用链：HTTP/业务服务 → internal/share.Create。失效原因：非正 TTL 会生成不可用分享或绕过平台的过期策略。证据：Create 根据 ttl 计算 ExpiresAt。 证据：Create 根据 ttl 计算 ExpiresAt。</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>目标行为：ttl&lt;=0 返回错误。边界：最小正 TTL可创建，过期后 Valid为false。合法场景：小时级或天级链接可访问。验证标准：无效参数错误非 nil，合法链接 Token 非空且未立即过期。</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-019/regression -count=1
+go test -race ./cases/bug-019/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>bug019_green</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>bug019_red</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Concurrent version creation must produce unique version identifiers for a document.</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>中文根因：版本创建的标识生成和写入必须在同一并发安全策略下执行。生产文件/符号：internal/document_version/repository.go:Repository.Create。失效原因：并发编辑生成重复 ID 会覆盖历史版本。证据：Create写入items并分配ID。 生产文件/符号：internal/document_version.Repository.Create 调用链：HTTP/业务服务 → internal/document_version.Repository.Create。失效原因：并发编辑生成重复 ID 会覆盖历史版本。证据：Create写入items并分配ID。 证据：Create写入items并分配ID。</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>目标行为：并发创建的版本 ID 全部唯一且记录数量完整。边界：同一文档和不同文档均适用。合法场景：多人协作自动保存产生多个版本。验证标准：race测试通过，ID集合大小等于创建数量。</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-020/regression -count=1
+go test -race ./cases/bug-020/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>bug020_green</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>bug020_red</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>diagnosis</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>context</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Expired recycle-bin cleanup must stop promptly when its context is cancelled.</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>中文根因：回收站批量清理属于后台任务，必须响应取消信号。生产文件/符号：internal/recycle/bin.go:PurgeExpired。失效原因：服务关闭时清理继续持锁会延迟退出。证据：PurgeExpired遍历并重建items切片。 生产文件/符号：internal/recycle.Bin.PurgeExpired 调用链：HTTP/业务服务 → internal/recycle.Bin.PurgeExpired。失效原因：服务关闭时清理继续持锁会延迟退出。证据：PurgeExpired遍历并重建items切片。 证据：PurgeExpired遍历并重建items切片。</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>目标行为：取消上下文返回0且不执行清理。边界：有效上下文清理过期项目，未过期项目保留。合法场景：定时任务在正常上下文运行。验证标准：取消调用不删除项目，有效调用只删除ExpiresAt早于now的项目。</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-021/regression -count=1
+go test -race ./cases/bug-021/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>bug021_green</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>bug021_red</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>diagnosis</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>nil</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Report generation must return a usable zero metric set when no activity exists.</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>中文根因：统计报表需要返回完整可序列化指标，而不是 nil 或未初始化结构。生产文件/符号：internal/report/report.go:Build。失效原因：看板读取空指针字段会导致页面渲染失败。证据：Build返回 Metrics并设置 GeneratedAt。 生产文件/符号：internal/report.Build 调用链：HTTP/业务服务 → internal/report.Build。失效原因：看板读取空指针字段会导致页面渲染失败。证据：Build返回 Metrics并设置 GeneratedAt。 证据：Build返回 Metrics并设置 GeneratedAt。</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>目标行为：空数据生成时间有效且所有数值为零。边界：取消上下文返回取消错误。合法场景：新空间无文档时仍可展示看板。验证标准：GeneratedAt非零，所有计数为零且无 panic。</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-022/regression -count=1
+go test -race ./cases/bug-022/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>bug022_green</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>bug022_red</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>diagnosis</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>slice</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Folder move validation must reject moving a folder into itself or any descendant.</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>中文根因：文件夹移动需要阻止环形父子关系。生产文件/符号：internal/folder/folder.go:CanMove。失效原因：形成循环后树遍历和权限继承会无限递归。证据：CanMove同时检查自身 ID和子路径前缀。 生产文件/符号：internal/folder.CanMove 调用链：HTTP/业务服务 → internal/folder.CanMove。失效原因：形成循环后树遍历和权限继承会无限递归。证据：CanMove同时检查自身 ID和子路径前缀。 证据：CanMove同时检查自身 ID和子路径前缀。</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>目标行为：自身和子孙目标均拒绝，其他目标允许。边界：空 ID不允许；同级兄弟目录可移动。合法场景：移动到根目录或其他分支。验证标准：布尔结果覆盖自身、子孙、合法目标和空值。</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-023/regression -count=1
+go test -race ./cases/bug-023/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>bug023_green</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>bug023_red</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>diagnosis</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Review decisions must reject unknown review IDs and preserve the record for valid decisions.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>中文根因：审核状态变更必须以存在的审核记录为前提。生产文件/符号：internal/review/service.go:Service.Decide。失效原因：错误 ID 被接受会造成文档状态与审核历史脱节。证据：Decide读取records并写回State、Opinion。 生产文件/符号：internal/review.Service.Decide 调用链：HTTP/业务服务 → internal/review.Service.Decide。失效原因：错误 ID 被接受会造成文档状态与审核历史脱节。证据：Decide读取records并写回State、Opinion。 证据：Decide读取records并写回State、Opinion。</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>目标行为：未知审核返回明确错误；已提交审核可被批准、驳回或退回。边界：状态值由审核状态枚举约束。合法场景：审核人处理pending记录。验证标准：错误包含 not found，合法决策保留同一 ID并更新意见。</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-024/regression -count=1
+go test -race ./cases/bug-024/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>bug024_green</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>bug024_red</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>bugfix</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Concurrent notification delivery must preserve every notification and mark only the target user read.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>中文根因：通知中心需要在并发写入和按用户读取之间保持数据一致性。生产文件/符号：internal/notification/center.go:Center.Push、MarkAllRead。失效原因：无锁或错误过滤会丢通知或误读其他用户消息。证据：Center维护共享items切片并提供按用户筛选。 生产文件/符号：internal/notification.Center.Push 调用链：HTTP/业务服务 → internal/notification.Center.Push。失效原因：无锁或错误过滤会丢通知或误读其他用户消息。证据：Center维护共享items切片并提供按用户筛选。 证据：Center维护共享items切片并提供按用户筛选。</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>目标行为：并发推送全部保留，标记用户A不影响用户B。边界：重复消息也应各自保留，空用户查询返回空。合法场景：评论、审核和发布事件同时推送。验证标准：race测试无竞争，用户计数准确，其他用户仍有未读通知。</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>go1.26.1 windows/amd64 (GOTOOLCHAIN=auto)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>go test ./cases/bug-025/regression -count=1
+go test -race ./cases/bug-025/regression -count=10</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>bug025_green</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>bug025_red</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>not uploaded</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:K11"/>
+  <autoFilter ref="A1:K26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
chore: record bug001 redgreen verification artifacts
</commit_message>
<xml_diff>
--- a/report-knowledge-asset-collaboration.xlsx
+++ b/report-knowledge-asset-collaboration.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="bug inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="verification" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'bug inventory'!$A$1:$K$26</definedName>
@@ -19,13 +20,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -48,8 +52,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -529,7 +534,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug01_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug01_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-001/packet-001.md</t>
         </is>
       </c>
     </row>
@@ -587,7 +592,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug02_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug02_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-002/packet-002.md</t>
         </is>
       </c>
     </row>
@@ -645,7 +650,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug03_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug03_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-003/packet-003.md</t>
         </is>
       </c>
     </row>
@@ -703,7 +708,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug04_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug04_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-004/packet-004.md</t>
         </is>
       </c>
     </row>
@@ -761,7 +766,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug05_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug05_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-005/packet-005.md</t>
         </is>
       </c>
     </row>
@@ -819,7 +824,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug06_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug06_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-006/packet-006.md</t>
         </is>
       </c>
     </row>
@@ -877,7 +882,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug07_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug07_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-007/packet-007.md</t>
         </is>
       </c>
     </row>
@@ -935,7 +940,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug08_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug08_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-008/packet-008.md</t>
         </is>
       </c>
     </row>
@@ -993,7 +998,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug09_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug09_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-009/packet-009.md</t>
         </is>
       </c>
     </row>
@@ -1051,7 +1056,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug10_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug10_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-010/packet-010.md</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1114,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug11_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug11_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-011/packet-011.md</t>
         </is>
       </c>
     </row>
@@ -1167,7 +1172,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug12_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug12_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-012/packet-012.md</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1230,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug13_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug13_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-013/packet-013.md</t>
         </is>
       </c>
     </row>
@@ -1283,7 +1288,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug14_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug14_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-014/packet-014.md</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1346,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug15_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug15_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-015/packet-015.md</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1404,7 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug16_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug16_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-016/packet-016.md</t>
         </is>
       </c>
     </row>
@@ -1457,7 +1462,7 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug17_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug17_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-017/packet-017.md</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1520,7 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug18_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug18_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-018/packet-018.md</t>
         </is>
       </c>
     </row>
@@ -1573,7 +1578,7 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug19_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug19_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-019/packet-019.md</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1636,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug20_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug20_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-020/packet-020.md</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1694,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug21_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug21_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-021/packet-021.md</t>
         </is>
       </c>
     </row>
@@ -1747,7 +1752,7 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug22_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug22_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-022/packet-022.md</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1810,7 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug23_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug23_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-023/packet-023.md</t>
         </is>
       </c>
     </row>
@@ -1863,7 +1868,7 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug24_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug24_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-024/packet-024.md</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1926,7 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>not uploaded</t>
+          <t>https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug25_green; https://github.com/zhangkui/knowledge-asset-collaboration/tree/bug25_red; https://github.com/zhangkui/knowledge-asset-collaboration/blob/master/cases/bug-025/packet-025.md</t>
         </is>
       </c>
     </row>
@@ -1929,4 +1934,172 @@
   <autoFilter ref="A1:K26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>production_go_files</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>production_go_lines</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5264</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>internal_tests</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>go_vet</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>gofmt</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>CLEAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>frontend_build</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>bug_packets_on_master</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>green_branches</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>red_branches</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>distinct_branch_tip_pairs</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>intentional_red_cases</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>003, 017, 019, 020</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>passing_cases</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>latest_master</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>3b675dd</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>